<commit_message>
Update map + table + spreadsheet
</commit_message>
<xml_diff>
--- a/co_courses.xlsx
+++ b/co_courses.xlsx
@@ -680,6 +680,9 @@
     <t>-106.817584</t>
   </si>
   <si>
+    <t>This course is so good, it gives CommonGround vibes, but with way closer mountains.</t>
+  </si>
+  <si>
     <t>Mountain Meadows Golf Club</t>
   </si>
   <si>
@@ -687,10 +690,6 @@
   </si>
   <si>
     <t>South Fork</t>
-  </si>
-  <si>
-    <t>40.791491
-</t>
   </si>
   <si>
     <r>
@@ -1856,10 +1855,6 @@
     <t>Avon</t>
   </si>
   <si>
-    <t>39.617870
-</t>
-  </si>
-  <si>
     <r>
       <rPr>
         <u val="single"/>
@@ -2214,6 +2209,9 @@
   </si>
   <si>
     <t>11/1/20</t>
+  </si>
+  <si>
+    <t xml:space="preserve">When I used to live in the Springs, I played here all the time. Fun little spot to grind on your wedges, best greens on a par 3 course. </t>
   </si>
   <si>
     <t>CommonGround Golf Course - Par 3</t>
@@ -4019,7 +4017,7 @@
     <xf numFmtId="59" fontId="0" fillId="4" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="15" fillId="4" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -4088,7 +4086,7 @@
     <xf numFmtId="14" fontId="0" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="6" fillId="4" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="61" fontId="0" fillId="4" borderId="7" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -6548,7 +6546,7 @@
       </c>
       <c r="N32" s="32"/>
     </row>
-    <row r="33" ht="59.8" customHeight="1">
+    <row r="33" ht="60.05" customHeight="1">
       <c r="A33" t="s" s="15">
         <v>177</v>
       </c>
@@ -6586,17 +6584,19 @@
       <c r="M33" s="29">
         <v>29</v>
       </c>
-      <c r="N33" s="33"/>
+      <c r="N33" t="s" s="25">
+        <v>182</v>
+      </c>
     </row>
     <row r="34" ht="248.35" customHeight="1">
       <c r="A34" t="s" s="15">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B34" t="s" s="16">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="C34" t="s" s="17">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D34" t="s" s="17">
         <v>25</v>
@@ -6604,8 +6604,8 @@
       <c r="E34" t="s" s="17">
         <v>37</v>
       </c>
-      <c r="F34" t="s" s="50">
-        <v>185</v>
+      <c r="F34" s="50">
+        <v>40.791491</v>
       </c>
       <c r="G34" s="18">
         <v>-105.575121</v>
@@ -10212,14 +10212,14 @@
       <c r="E122" t="s" s="17">
         <v>37</v>
       </c>
-      <c r="F122" t="s" s="73">
-        <v>495</v>
+      <c r="F122" s="73">
+        <v>39.61787</v>
       </c>
       <c r="G122" s="18">
         <v>-106.476058</v>
       </c>
       <c r="H122" t="s" s="31">
-        <v>496</v>
+        <v>495</v>
       </c>
       <c r="I122" t="s" s="51">
         <v>126</v>
@@ -10240,10 +10240,10 @@
     </row>
     <row r="123" ht="44.8" customHeight="1">
       <c r="A123" t="s" s="15">
+        <v>496</v>
+      </c>
+      <c r="B123" t="s" s="16">
         <v>497</v>
-      </c>
-      <c r="B123" t="s" s="16">
-        <v>498</v>
       </c>
       <c r="C123" t="s" s="17">
         <v>147</v>
@@ -10264,7 +10264,7 @@
         <v>27</v>
       </c>
       <c r="I123" t="s" s="39">
-        <v>499</v>
+        <v>498</v>
       </c>
       <c r="J123" s="40">
         <v>101</v>
@@ -10282,7 +10282,7 @@
     </row>
     <row r="124" ht="59.8" customHeight="1">
       <c r="A124" t="s" s="15">
-        <v>500</v>
+        <v>499</v>
       </c>
       <c r="B124" t="s" s="16">
         <v>438</v>
@@ -10322,7 +10322,7 @@
     </row>
     <row r="125" ht="59.8" customHeight="1">
       <c r="A125" t="s" s="15">
-        <v>501</v>
+        <v>500</v>
       </c>
       <c r="B125" t="s" s="16">
         <v>438</v>
@@ -10346,7 +10346,7 @@
         <v>27</v>
       </c>
       <c r="I125" t="s" s="39">
-        <v>502</v>
+        <v>501</v>
       </c>
       <c r="J125" s="40">
         <v>92</v>
@@ -10364,13 +10364,13 @@
     </row>
     <row r="126" ht="44.8" customHeight="1">
       <c r="A126" t="s" s="15">
+        <v>502</v>
+      </c>
+      <c r="B126" t="s" s="16">
         <v>503</v>
       </c>
-      <c r="B126" t="s" s="16">
+      <c r="C126" t="s" s="17">
         <v>504</v>
-      </c>
-      <c r="C126" t="s" s="17">
-        <v>505</v>
       </c>
       <c r="D126" t="s" s="17">
         <v>25</v>
@@ -10388,7 +10388,7 @@
         <v>27</v>
       </c>
       <c r="I126" t="s" s="39">
-        <v>506</v>
+        <v>505</v>
       </c>
       <c r="J126" s="40">
         <v>94</v>
@@ -10406,10 +10406,10 @@
     </row>
     <row r="127" ht="44.8" customHeight="1">
       <c r="A127" t="s" s="15">
+        <v>506</v>
+      </c>
+      <c r="B127" t="s" s="16">
         <v>507</v>
-      </c>
-      <c r="B127" t="s" s="16">
-        <v>508</v>
       </c>
       <c r="C127" t="s" s="17">
         <v>24</v>
@@ -10430,7 +10430,7 @@
         <v>27</v>
       </c>
       <c r="I127" t="s" s="39">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="J127" s="40">
         <v>103</v>
@@ -10448,10 +10448,10 @@
     </row>
     <row r="128" ht="102.35" customHeight="1">
       <c r="A128" t="s" s="15">
+        <v>509</v>
+      </c>
+      <c r="B128" t="s" s="16">
         <v>510</v>
-      </c>
-      <c r="B128" t="s" s="16">
-        <v>511</v>
       </c>
       <c r="C128" t="s" s="17">
         <v>201</v>
@@ -10470,7 +10470,7 @@
       </c>
       <c r="H128" s="33"/>
       <c r="I128" t="s" s="20">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="J128" s="21">
         <v>35</v>
@@ -10483,15 +10483,15 @@
         <v>126</v>
       </c>
       <c r="N128" t="s" s="30">
-        <v>513</v>
+        <v>512</v>
       </c>
     </row>
     <row r="129" ht="59.8" customHeight="1">
       <c r="A129" t="s" s="15">
+        <v>513</v>
+      </c>
+      <c r="B129" t="s" s="16">
         <v>514</v>
-      </c>
-      <c r="B129" t="s" s="16">
-        <v>515</v>
       </c>
       <c r="C129" t="s" s="17">
         <v>205</v>
@@ -10530,10 +10530,10 @@
     </row>
     <row r="130" ht="44.8" customHeight="1">
       <c r="A130" t="s" s="15">
+        <v>515</v>
+      </c>
+      <c r="B130" t="s" s="16">
         <v>516</v>
-      </c>
-      <c r="B130" t="s" s="16">
-        <v>517</v>
       </c>
       <c r="C130" t="s" s="17">
         <v>152</v>
@@ -10554,7 +10554,7 @@
         <v>27</v>
       </c>
       <c r="I130" t="s" s="39">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J130" s="40">
         <v>96</v>
@@ -10572,10 +10572,10 @@
     </row>
     <row r="131" ht="340.35" customHeight="1">
       <c r="A131" t="s" s="15">
+        <v>518</v>
+      </c>
+      <c r="B131" t="s" s="16">
         <v>519</v>
-      </c>
-      <c r="B131" t="s" s="16">
-        <v>520</v>
       </c>
       <c r="C131" t="s" s="17">
         <v>49</v>
@@ -10594,7 +10594,7 @@
       </c>
       <c r="H131" s="33"/>
       <c r="I131" t="s" s="20">
-        <v>521</v>
+        <v>520</v>
       </c>
       <c r="J131" s="21">
         <v>13</v>
@@ -10609,15 +10609,15 @@
         <v>129</v>
       </c>
       <c r="N131" t="s" s="30">
-        <v>522</v>
+        <v>521</v>
       </c>
     </row>
     <row r="132" ht="59.8" customHeight="1">
       <c r="A132" t="s" s="15">
+        <v>522</v>
+      </c>
+      <c r="B132" t="s" s="16">
         <v>523</v>
-      </c>
-      <c r="B132" t="s" s="16">
-        <v>524</v>
       </c>
       <c r="C132" t="s" s="17">
         <v>135</v>
@@ -10654,13 +10654,13 @@
     </row>
     <row r="133" ht="44.8" customHeight="1">
       <c r="A133" t="s" s="15">
+        <v>524</v>
+      </c>
+      <c r="B133" t="s" s="16">
         <v>525</v>
       </c>
-      <c r="B133" t="s" s="16">
+      <c r="C133" t="s" s="17">
         <v>526</v>
-      </c>
-      <c r="C133" t="s" s="17">
-        <v>527</v>
       </c>
       <c r="D133" t="s" s="17">
         <v>25</v>
@@ -10675,10 +10675,10 @@
         <v>-102.8043</v>
       </c>
       <c r="H133" t="s" s="31">
+        <v>527</v>
+      </c>
+      <c r="I133" t="s" s="51">
         <v>528</v>
-      </c>
-      <c r="I133" t="s" s="51">
-        <v>529</v>
       </c>
       <c r="J133" s="52">
         <v>127</v>
@@ -10696,13 +10696,13 @@
     </row>
     <row r="134" ht="29.8" customHeight="1">
       <c r="A134" t="s" s="15">
+        <v>529</v>
+      </c>
+      <c r="B134" t="s" s="16">
         <v>530</v>
       </c>
-      <c r="B134" t="s" s="16">
+      <c r="C134" t="s" s="17">
         <v>531</v>
-      </c>
-      <c r="C134" t="s" s="17">
-        <v>532</v>
       </c>
       <c r="D134" t="s" s="17">
         <v>25</v>
@@ -10711,13 +10711,13 @@
         <v>37</v>
       </c>
       <c r="F134" t="s" s="35">
+        <v>532</v>
+      </c>
+      <c r="G134" t="s" s="35">
         <v>533</v>
       </c>
-      <c r="G134" t="s" s="35">
+      <c r="H134" t="s" s="25">
         <v>534</v>
-      </c>
-      <c r="H134" t="s" s="25">
-        <v>535</v>
       </c>
       <c r="I134" s="59">
         <v>46208</v>
@@ -10738,13 +10738,13 @@
     </row>
     <row r="135" ht="59.8" customHeight="1">
       <c r="A135" t="s" s="15">
+        <v>535</v>
+      </c>
+      <c r="B135" t="s" s="16">
         <v>536</v>
       </c>
-      <c r="B135" t="s" s="16">
+      <c r="C135" t="s" s="17">
         <v>537</v>
-      </c>
-      <c r="C135" t="s" s="17">
-        <v>538</v>
       </c>
       <c r="D135" t="s" s="17">
         <v>25</v>
@@ -10760,7 +10760,7 @@
       </c>
       <c r="H135" s="33"/>
       <c r="I135" t="s" s="20">
-        <v>539</v>
+        <v>538</v>
       </c>
       <c r="J135" s="21">
         <v>62</v>
@@ -10778,10 +10778,10 @@
     </row>
     <row r="136" ht="44.8" customHeight="1">
       <c r="A136" t="s" s="15">
+        <v>539</v>
+      </c>
+      <c r="B136" t="s" s="16">
         <v>540</v>
-      </c>
-      <c r="B136" t="s" s="16">
-        <v>541</v>
       </c>
       <c r="C136" t="s" s="17">
         <v>24</v>
@@ -10793,10 +10793,10 @@
         <v>26</v>
       </c>
       <c r="F136" t="s" s="35">
+        <v>541</v>
+      </c>
+      <c r="G136" t="s" s="35">
         <v>542</v>
-      </c>
-      <c r="G136" t="s" s="35">
-        <v>543</v>
       </c>
       <c r="H136" s="33"/>
       <c r="I136" s="74">
@@ -10818,13 +10818,13 @@
     </row>
     <row r="137" ht="44.8" customHeight="1">
       <c r="A137" t="s" s="15">
+        <v>543</v>
+      </c>
+      <c r="B137" t="s" s="16">
         <v>544</v>
       </c>
-      <c r="B137" t="s" s="16">
+      <c r="C137" t="s" s="17">
         <v>545</v>
-      </c>
-      <c r="C137" t="s" s="17">
-        <v>546</v>
       </c>
       <c r="D137" t="s" s="17">
         <v>25</v>
@@ -10839,7 +10839,7 @@
         <v>-105.760061</v>
       </c>
       <c r="H137" t="s" s="25">
-        <v>547</v>
+        <v>546</v>
       </c>
       <c r="I137" s="26">
         <v>46208</v>
@@ -10860,13 +10860,13 @@
     </row>
     <row r="138" ht="44.8" customHeight="1">
       <c r="A138" t="s" s="15">
+        <v>547</v>
+      </c>
+      <c r="B138" t="s" s="16">
         <v>548</v>
       </c>
-      <c r="B138" t="s" s="16">
+      <c r="C138" t="s" s="17">
         <v>549</v>
-      </c>
-      <c r="C138" t="s" s="17">
-        <v>550</v>
       </c>
       <c r="D138" t="s" s="17">
         <v>25</v>
@@ -10884,7 +10884,7 @@
         <v>27</v>
       </c>
       <c r="I138" t="s" s="39">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="J138" s="40">
         <v>106</v>
@@ -10902,13 +10902,13 @@
     </row>
     <row r="139" ht="44.8" customHeight="1">
       <c r="A139" t="s" s="15">
+        <v>551</v>
+      </c>
+      <c r="B139" t="s" s="16">
         <v>552</v>
       </c>
-      <c r="B139" t="s" s="16">
+      <c r="C139" t="s" s="17">
         <v>553</v>
-      </c>
-      <c r="C139" t="s" s="17">
-        <v>554</v>
       </c>
       <c r="D139" t="s" s="17">
         <v>25</v>
@@ -10926,7 +10926,7 @@
         <v>27</v>
       </c>
       <c r="I139" t="s" s="39">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="J139" s="40">
         <v>108</v>
@@ -10944,13 +10944,13 @@
     </row>
     <row r="140" ht="44.8" customHeight="1">
       <c r="A140" t="s" s="15">
+        <v>554</v>
+      </c>
+      <c r="B140" t="s" s="16">
         <v>555</v>
       </c>
-      <c r="B140" t="s" s="16">
+      <c r="C140" t="s" s="17">
         <v>556</v>
-      </c>
-      <c r="C140" t="s" s="17">
-        <v>557</v>
       </c>
       <c r="D140" t="s" s="17">
         <v>25</v>
@@ -10959,13 +10959,13 @@
         <v>50</v>
       </c>
       <c r="F140" t="s" s="35">
+        <v>557</v>
+      </c>
+      <c r="G140" t="s" s="35">
         <v>558</v>
       </c>
-      <c r="G140" t="s" s="35">
+      <c r="H140" t="s" s="25">
         <v>559</v>
-      </c>
-      <c r="H140" t="s" s="25">
-        <v>560</v>
       </c>
       <c r="I140" s="26">
         <v>46209</v>
@@ -10986,10 +10986,10 @@
     </row>
     <row r="141" ht="154.35" customHeight="1">
       <c r="A141" t="s" s="15">
+        <v>560</v>
+      </c>
+      <c r="B141" t="s" s="16">
         <v>561</v>
-      </c>
-      <c r="B141" t="s" s="16">
-        <v>562</v>
       </c>
       <c r="C141" t="s" s="17">
         <v>209</v>
@@ -11007,7 +11007,7 @@
         <v>-105.33581</v>
       </c>
       <c r="H141" t="s" s="25">
-        <v>563</v>
+        <v>562</v>
       </c>
       <c r="I141" s="59">
         <v>46202</v>
@@ -11025,15 +11025,15 @@
         <v>140</v>
       </c>
       <c r="N141" t="s" s="30">
-        <v>564</v>
+        <v>563</v>
       </c>
     </row>
     <row r="142" ht="44.8" customHeight="1">
       <c r="A142" t="s" s="15">
-        <v>565</v>
+        <v>564</v>
       </c>
       <c r="B142" t="s" s="16">
-        <v>517</v>
+        <v>516</v>
       </c>
       <c r="C142" t="s" s="17">
         <v>152</v>
@@ -11054,7 +11054,7 @@
         <v>27</v>
       </c>
       <c r="I142" t="s" s="39">
-        <v>518</v>
+        <v>517</v>
       </c>
       <c r="J142" s="40">
         <v>95</v>
@@ -11072,10 +11072,10 @@
     </row>
     <row r="143" ht="44.8" customHeight="1">
       <c r="A143" t="s" s="15">
+        <v>565</v>
+      </c>
+      <c r="B143" t="s" s="16">
         <v>566</v>
-      </c>
-      <c r="B143" t="s" s="16">
-        <v>567</v>
       </c>
       <c r="C143" t="s" s="17">
         <v>16</v>
@@ -11093,10 +11093,10 @@
         <v>-102.3025</v>
       </c>
       <c r="H143" t="s" s="31">
+        <v>567</v>
+      </c>
+      <c r="I143" t="s" s="51">
         <v>568</v>
-      </c>
-      <c r="I143" t="s" s="51">
-        <v>569</v>
       </c>
       <c r="J143" s="52">
         <v>126</v>
@@ -11114,7 +11114,7 @@
     </row>
     <row r="144" ht="44.8" customHeight="1">
       <c r="A144" t="s" s="15">
-        <v>570</v>
+        <v>569</v>
       </c>
       <c r="B144" t="s" s="16">
         <v>355</v>
@@ -11135,10 +11135,10 @@
         <v>-104.939592</v>
       </c>
       <c r="H144" t="s" s="31">
+        <v>570</v>
+      </c>
+      <c r="I144" t="s" s="51">
         <v>571</v>
-      </c>
-      <c r="I144" t="s" s="51">
-        <v>572</v>
       </c>
       <c r="J144" s="52">
         <v>128</v>
@@ -11154,9 +11154,9 @@
       </c>
       <c r="N144" s="67"/>
     </row>
-    <row r="145" ht="59.8" customHeight="1">
+    <row r="145" ht="112.05" customHeight="1">
       <c r="A145" t="s" s="15">
-        <v>573</v>
+        <v>572</v>
       </c>
       <c r="B145" t="s" s="16">
         <v>476</v>
@@ -11178,7 +11178,7 @@
       </c>
       <c r="H145" s="33"/>
       <c r="I145" t="s" s="20">
-        <v>574</v>
+        <v>573</v>
       </c>
       <c r="J145" s="21">
         <v>21</v>
@@ -11192,7 +11192,9 @@
       <c r="M145" s="37">
         <v>144</v>
       </c>
-      <c r="N145" s="33"/>
+      <c r="N145" t="s" s="25">
+        <v>574</v>
+      </c>
     </row>
     <row r="146" ht="44.8" customHeight="1">
       <c r="A146" t="s" s="15">
@@ -11388,7 +11390,7 @@
         <v>27</v>
       </c>
       <c r="I150" t="s" s="39">
-        <v>551</v>
+        <v>550</v>
       </c>
       <c r="J150" s="40">
         <v>107</v>
@@ -12110,7 +12112,7 @@
         <v>636</v>
       </c>
       <c r="C170" t="s" s="17">
-        <v>546</v>
+        <v>545</v>
       </c>
       <c r="D170" t="s" s="17">
         <v>25</v>
@@ -13305,7 +13307,7 @@
         <v>712</v>
       </c>
       <c r="B203" t="s" s="16">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="C203" t="s" s="17">
         <v>24</v>
@@ -13341,7 +13343,7 @@
         <v>713</v>
       </c>
       <c r="B204" t="s" s="16">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="C204" t="s" s="17">
         <v>24</v>
@@ -15432,7 +15434,7 @@
         <v>842</v>
       </c>
       <c r="C262" t="s" s="17">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="D262" t="s" s="17">
         <v>17</v>

</xml_diff>